<commit_message>
Selfi printer v1: kabinet efter DNP's vejledning og fotos
Papirudgangen sidder ca. 135 mm over printerens bund (var 46), så slids og bakke er flyttet op og logoet ned under bakken. Pi'en får strøm fra printerens 5 V 2 A USB-udgang, så 5 V-forsyning og Y-kabel er væk. Udluftning i begge sider ud for printerens blæser. Vinklede C13- og USB-B-stik i bagrummet.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KS5yd6iUQhhKJ7JKEceAzD
</commit_message>
<xml_diff>
--- a/hardware/stl/printer/selfi-printer-v1/selfi-printer-v1_indkoebsliste.xlsx
+++ b/hardware/stl/printer/selfi-printer-v1/selfi-printer-v1_indkoebsliste.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -546,7 +546,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Skøn; til fotostriber 2×6. Bekræft at den sælges i EU</t>
+          <t>Skøn; til fotostriber 2×6, kræver firmware v1.10 + ny driver. Bekræft at den sælges i EU</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>USB-kabel micro-USB (OTG) → USB-B, 30 cm</t>
+          <t>USB-kabel micro-USB (OTG) → USB-B vinklet, 30 cm</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -620,14 +620,14 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Pi Zero → printer</t>
+          <t>Pi Zero (USB) → printerens USB-B; vinklet stik, bagrummet er 40 mm</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mean Well GST25E05-P1J, 5 V 4 A (C8-indgang)</t>
+          <t>USB-kabel USB-A → micro-USB, 20 cm</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -639,21 +639,21 @@
         <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>160</v>
+        <v>30</v>
       </c>
       <c r="E10" t="n">
-        <v>160</v>
+        <v>30</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Strøm til Pi'en</t>
+          <t>Printerens 5 V 2 A-udgang → Pi Zero (PWR-stik); ingen ekstra forsyning</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Adapterkabel DC 5,5/2,1 hun → micro-USB, 15 cm</t>
+          <t>Panelkabel C14 snap-in → C13 vinklet, 30 cm</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -665,21 +665,21 @@
         <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="E11" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Forsyning → Pi Zero (PWR-stik)</t>
+          <t>Strømindgang i soklen → printerens C14-stik bagpå</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Panelkabel C14 snap-in → C13, 30 cm</t>
+          <t>Strømkabel Schuko → C13, 2 m</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -691,21 +691,21 @@
         <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="E12" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Strømindgang i soklen bagpå</t>
+          <t>Det eneste kabel kunden sætter i</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Y-kabel C14 → C13 + C7, 30 cm</t>
+          <t>Gummifødder Ø12 × 1 mm, selvklæbende</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -714,212 +714,212 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>60</v>
+        <v>5</v>
       </c>
       <c r="E13" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Printer (C13, tjekkes) + forsyning (C8)</t>
+          <t>I fordybningerne under soklen</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Strømkabel Schuko → C13, 2 m</t>
+          <t>Skabslås / kamlås Ø19, cylinder til plade op til 12 mm, med kam</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Alle</t>
+          <t>B2B</t>
         </is>
       </c>
       <c r="C14" t="n">
         <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="E14" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Det eneste kabel kunden sætter i</t>
+          <t>Samme nøgle til alle steder</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Gummifødder Ø12 × 1 mm, selvklæbende</t>
+          <t>SPUN+ Climate 4,0 × 30, undersænket</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Alle</t>
+          <t>B2B</t>
         </is>
       </c>
       <c r="C15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" t="n">
         <v>4</v>
       </c>
-      <c r="D15" t="n">
-        <v>5</v>
-      </c>
-      <c r="E15" t="n">
-        <v>20</v>
-      </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>I fordybningerne under soklen</t>
+          <t>Sokkel → hylde eller konsol</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Skabslås / kamlås Ø19, cylinder til plade op til 12 mm, med kam</t>
+          <t>Skrue 5 × 50 + Fischer DuoPower 8 × 40</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>B2B</t>
+          <t>B2B væg</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D16" t="n">
-        <v>60</v>
+        <v>4</v>
       </c>
       <c r="E16" t="n">
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Samme nøgle til alle steder</t>
+          <t>Vægplade → væg (stedet monterer selv)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SPUN+ Climate 4,0 × 30, undersænket</t>
+          <t>Låseskrue DIN 7982 pin-Torx 4,2 × 25</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>B2B</t>
+          <t>B2B væg</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Sokkel → hylde eller konsol</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Skrue 5 × 50 + Fischer DuoPower 8 × 40</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>B2B væg</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>4</v>
-      </c>
-      <c r="D18" t="n">
-        <v>4</v>
-      </c>
-      <c r="E18" t="n">
-        <v>16</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Vægplade → væg (stedet monterer selv)</t>
+          <t>Konsol → vægplade (som gen 2)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Låseskrue DIN 7982 pin-Torx 4,2 × 25</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>B2B væg</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" t="n">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Printede dele (ASA)</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Bruges til</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Gram</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Kr pr. g</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>I alt</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Farve</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Kappe (B2C) eller kappe med låsehul (B2B)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Alle</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>900</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E20" t="n">
+        <v>225</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>sort ASA</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Logo, hvide dele + grønne prikker (indlagt i kappen)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Alle</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
         <v>3</v>
       </c>
-      <c r="E19" t="n">
-        <v>3</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Konsol → vægplade (som gen 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Printede dele (ASA)</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Bruges til</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Gram</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Kr pr. g</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>I alt</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>Farve</t>
+      <c r="D21" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>hvid + grøn ASA</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Kappe (B2C) eller kappe med låsehul (B2B)</t>
+          <t>Sokkel</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>900</v>
+        <v>420</v>
       </c>
       <c r="D22" t="n">
         <v>0.25</v>
       </c>
       <c r="E22" t="n">
-        <v>225</v>
+        <v>105</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -945,7 +945,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Logo, hvide dele + grønne prikker (indlagt i kappen)</t>
+          <t>Opsamlingsbakke</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -954,39 +954,39 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>60</v>
       </c>
       <c r="D23" t="n">
         <v>0.25</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>hvid + grøn ASA</t>
+          <t>sort ASA</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Sokkel</t>
+          <t>Vægkonsol</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Alle</t>
+          <t>B2B væg</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>420</v>
+        <v>700</v>
       </c>
       <c r="D24" t="n">
         <v>0.25</v>
       </c>
       <c r="E24" t="n">
-        <v>105</v>
+        <v>175</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -997,22 +997,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Opsamlingsbakke</t>
+          <t>Vægplade</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Alle</t>
+          <t>B2B væg</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>60</v>
+        <v>220</v>
       </c>
       <c r="D25" t="n">
         <v>0.25</v>
       </c>
       <c r="E25" t="n">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1020,119 +1020,67 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Vægkonsol</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>B2B væg</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>700</v>
-      </c>
-      <c r="D26" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E26" t="n">
-        <v>175</v>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>sort ASA</t>
-        </is>
-      </c>
-    </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Vægplade</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>B2B væg</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>220</v>
-      </c>
-      <c r="D27" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E27" t="n">
-        <v>55</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>sort ASA</t>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Sum</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Printer-pakke B2C (bord)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="n">
+        <v>9296</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>inkl. begge ruller</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>Sum</t>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>B2B hylde/disk</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
+      <c r="E29" t="n">
+        <v>9360</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>+ lås og 2 skruer</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Printer-pakke B2C (bord)</t>
+          <t>B2B væg</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="n">
-        <v>9516</v>
+        <v>9609</v>
       </c>
       <c r="F30" t="inlineStr">
-        <is>
-          <t>inkl. begge ruller</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>B2B hylde/disk</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="n">
-        <v>9580</v>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>+ lås og 2 skruer</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>B2B væg</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="n">
-        <v>9829</v>
-      </c>
-      <c r="F32" t="inlineStr">
         <is>
           <t>+ konsol, vægplade og skruer</t>
         </is>

</xml_diff>